<commit_message>
Planificacion julio y agosto 2026 + mejoras al motor
- Motor: arrastre de saldo acumulado entre meses (lee saldo del mes anterior)
- Motor: tope blando (si no entra en el presupuesto, relaja y arrastra la deuda)
- Correccion mayo: quitadas 4 rutas no hechas; saldos may/jun a acumulado
- Planificacion julio (bencina 1496, 22 dias) y agosto (21 dias)
- Nuevos scripts: generar_limites_excel.py, generar_paso_a_paso.py
- generar_limites_excel acepta mes por numero o nombre
- HANDOFF.md con el estado y traspaso del proyecto
- .gitignore: ignora temporales de Excel (~$)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/Rutas__Kilometros_Auditores.xlsx
+++ b/app/Rutas__Kilometros_Auditores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6a51e5493e413da3/Desktop/Seguros Digitales/2.- El Roble - Coca Cola/Planificación Logistica/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valen\Documents\Prieto_Correa_seguros\coca_cola\Modelo_Coca-Cola\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_A8D2F9357183CDBFAC99A5931297BF8D13263215" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F384F76-58DB-47B7-ACA7-C6AE69C6E8B2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3169BC94-A2BE-4729-838D-285973419064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="918" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="918" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carlos Acevedo" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cristian Lizama'!$B$3:$D$58</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Samuel Inostroza'!$B$3:$D$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mauricio Picart'!$B$3:$D$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Samuel Inostroza'!$B$3:$G$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="227">
   <si>
     <t>Universidad de Talca</t>
   </si>
@@ -394,329 +395,344 @@
     <t>Padre Hurtado</t>
   </si>
   <si>
+    <t>Villa la Paz</t>
+  </si>
+  <si>
+    <t>Cancha Rayada</t>
+  </si>
+  <si>
+    <t>Aurora de Chile</t>
+  </si>
+  <si>
+    <t>Villa Perú</t>
+  </si>
+  <si>
+    <t>Linares: Pob. La 35</t>
+  </si>
+  <si>
+    <t>Linares: San Antonio</t>
+  </si>
+  <si>
+    <t>Linares: Salida Cuellar</t>
+  </si>
+  <si>
+    <t>Linares: Villa Alegre</t>
+  </si>
+  <si>
+    <t>Linares: Melozal</t>
+  </si>
+  <si>
+    <t>Linares: Palmilla</t>
+  </si>
+  <si>
+    <t>Linares: El Esfuerzo</t>
+  </si>
+  <si>
+    <t>Linares: Salida Huapi</t>
+  </si>
+  <si>
+    <t>Iloca - Duao - Lipimavida</t>
+  </si>
+  <si>
+    <t>Llico - Vichuquen</t>
+  </si>
+  <si>
+    <t>Licantén</t>
+  </si>
+  <si>
+    <t>Curepto</t>
+  </si>
+  <si>
+    <t>Lora - Curepto</t>
+  </si>
+  <si>
+    <t>Palquibudi - La Huerta</t>
+  </si>
+  <si>
+    <t>Hualañe</t>
+  </si>
+  <si>
+    <t>Centro Plaza</t>
+  </si>
+  <si>
+    <t>Lontue - Sagrada Familia</t>
+  </si>
+  <si>
+    <t>Carretera Rauquen - Avda. España</t>
+  </si>
+  <si>
+    <t>Lontue - Pichingal - Casa Blanca</t>
+  </si>
+  <si>
+    <t>Romeral - Los Guaicos</t>
+  </si>
+  <si>
+    <t>Los Niches</t>
+  </si>
+  <si>
+    <t>Villa Prat - Sagrada Familia</t>
+  </si>
+  <si>
+    <t>Sol de Septiembre - Manuel Rodríguez</t>
+  </si>
+  <si>
+    <t>Feria - Mall - Terminal</t>
+  </si>
+  <si>
+    <t>Guaiquillo - Aguas Negras</t>
+  </si>
+  <si>
+    <t>Hospital - Alameda - Mataquito</t>
+  </si>
+  <si>
+    <t>Rauco - Comalle</t>
+  </si>
+  <si>
+    <t>Itahue Molina Estación</t>
+  </si>
+  <si>
+    <t>El Boldo</t>
+  </si>
+  <si>
+    <t>Bombero Garrido - Vaticano</t>
+  </si>
+  <si>
+    <t>La Montaña - Teno - Viluco</t>
+  </si>
+  <si>
+    <t>Santa Fe</t>
+  </si>
+  <si>
+    <t>Aguas Negras</t>
+  </si>
+  <si>
+    <t>Teno - Arboleda</t>
+  </si>
+  <si>
+    <t>Sarmiento - Rauquen</t>
+  </si>
+  <si>
+    <t>Molina Centro Porvenir</t>
+  </si>
+  <si>
+    <t>Bombero Garrido - Tutuquen</t>
+  </si>
+  <si>
+    <t>Santa Lucia - Santos Martínez</t>
+  </si>
+  <si>
+    <t>CURICÓ</t>
+  </si>
+  <si>
+    <t>Auditor : SAMUEL INOSTROZA NAVARRO</t>
+  </si>
+  <si>
+    <t>Linares: Obispo Camus - Yerbas Buenas</t>
+  </si>
+  <si>
+    <t>Auditor : CRISTIAN LIZAMA VERGARA</t>
+  </si>
+  <si>
+    <t>SAN FDO</t>
+  </si>
+  <si>
+    <t>ANGOSTURA -  18 DE SEPTIEMBRE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APALTA - PANIAHUE </t>
+  </si>
+  <si>
+    <t>AUQUINCO - PUJILLAY</t>
+  </si>
+  <si>
+    <t>CALLEJONES - NANCAGUA</t>
+  </si>
+  <si>
+    <t>CHEPICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHEPICA - LAS ALAMEDAS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHEPICA - QUINAHUE </t>
+  </si>
+  <si>
+    <t>CHIMBARONGO  CENTRO</t>
+  </si>
+  <si>
+    <t>CHIMBARONGO CENTRO PTE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHIMBARONGO NORTE </t>
+  </si>
+  <si>
+    <t>CHIMBARONGO NORTE -CENTRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHIMBARONGO SUR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CODEGUA - PEOR ES NADA </t>
+  </si>
+  <si>
+    <t>CUNACO- CRUCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL HHUIQUE - PERALILLO </t>
+  </si>
+  <si>
+    <t>LOLOL - LA LAJUELA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARCGIHUE </t>
+  </si>
+  <si>
+    <t>NANCAGUA -CENTRO</t>
+  </si>
+  <si>
+    <t>NANCAGUA - SAN GREGORIO</t>
+  </si>
+  <si>
+    <t>PAREDONES - LOLOL</t>
+  </si>
+  <si>
+    <t>PERALILLO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PICHILEMU -ALCONES </t>
+  </si>
+  <si>
+    <t>POICHILEMU - AV.CAHUIL</t>
+  </si>
+  <si>
+    <t>PICHILEMU - CENTRO</t>
+  </si>
+  <si>
+    <t>PICHILEMU - COSTANERA</t>
+  </si>
+  <si>
+    <t>PICHILEMU - INFIERNILLO</t>
+  </si>
+  <si>
+    <t>PICHILEMU - ORIENTE</t>
+  </si>
+  <si>
+    <t>PLACILLA</t>
+  </si>
+  <si>
+    <t>POBLACION - PERALILLO</t>
+  </si>
+  <si>
+    <t>PUENTE NEGRO - AGUA BUENA</t>
+  </si>
+  <si>
+    <t>PUMANQUE - NILAHUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROMA - MIRAFLORES -POLONIA </t>
+  </si>
+  <si>
+    <t>ROMERAL - SAN JUAN - TINGURIRICA</t>
+  </si>
+  <si>
+    <t>SAN FDO. - CENTINELA</t>
+  </si>
+  <si>
+    <t>SAN FDO. - CENTRO</t>
+  </si>
+  <si>
+    <t>SAN FDO. CENTRO 2</t>
+  </si>
+  <si>
+    <t>SAN FDO. CENTRO - PLAZA</t>
+  </si>
+  <si>
+    <t>SAN FDO. - MANSO DE VELASCO</t>
+  </si>
+  <si>
+    <t>SAN FDO, - GABRIELA MISTRAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAN FDO. - INDEPENDENCIA </t>
+  </si>
+  <si>
+    <t>SAN FDO. - NOR PONIENTE</t>
+  </si>
+  <si>
+    <t>SAN FDO. - ORIENTE</t>
+  </si>
+  <si>
+    <t>SAN FDO.  -SAN HERNAN</t>
+  </si>
+  <si>
+    <t>SAN FDO SUR</t>
+  </si>
+  <si>
+    <t>SAN  FDO. - SUR PONIENTE</t>
+  </si>
+  <si>
+    <t>SAN FDO. SUR PONIENTE 2</t>
+  </si>
+  <si>
+    <t>SAN FDO. TERMINAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STA CRUZ  - AV. ERRAZURIZ </t>
+  </si>
+  <si>
+    <t>STA CRUZ - BARREALES - PALMILLA</t>
+  </si>
+  <si>
+    <t>SATA .CRUZ ORIENTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STA CRUZ PONIENTE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">STA CRUZ SUR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">STA CRUZ TERMINAL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VILLA ALEGRE - LA TUNA </t>
+  </si>
+  <si>
+    <t>CANT</t>
+  </si>
+  <si>
     <t>Don Gonzalo</t>
   </si>
   <si>
-    <t>Villa la Paz</t>
-  </si>
-  <si>
-    <t>Cancha Rayada</t>
-  </si>
-  <si>
-    <t>Aurora de Chile</t>
-  </si>
-  <si>
-    <t>Villa Perú</t>
-  </si>
-  <si>
-    <t>Linares: Pob. La 35</t>
-  </si>
-  <si>
-    <t>Linares: San Antonio</t>
-  </si>
-  <si>
-    <t>Linares: Salida Cuellar</t>
-  </si>
-  <si>
     <t>Linares: Centro Sur Linares</t>
   </si>
   <si>
-    <t>Linares: Villa Alegre</t>
-  </si>
-  <si>
     <t>Linares: Villa Alegre Centro</t>
   </si>
   <si>
-    <t>Linares: Melozal</t>
-  </si>
-  <si>
-    <t>Linares: Palmilla</t>
-  </si>
-  <si>
-    <t>Linares: El Esfuerzo</t>
-  </si>
-  <si>
-    <t>Linares: Salida Huapi</t>
-  </si>
-  <si>
     <t>Linares: Centro Brasil</t>
   </si>
   <si>
-    <t>Iloca - Duao - Lipimavida</t>
-  </si>
-  <si>
-    <t>Llico - Vichuquen</t>
-  </si>
-  <si>
-    <t>Licantén</t>
-  </si>
-  <si>
-    <t>Curepto</t>
-  </si>
-  <si>
-    <t>Lora - Curepto</t>
-  </si>
-  <si>
-    <t>Palquibudi - La Huerta</t>
-  </si>
-  <si>
-    <t>Hualañe</t>
-  </si>
-  <si>
-    <t>Centro Plaza</t>
-  </si>
-  <si>
-    <t>Lontue - Sagrada Familia</t>
-  </si>
-  <si>
-    <t>Carretera Rauquen - Avda. España</t>
-  </si>
-  <si>
-    <t>Lontue - Pichingal - Casa Blanca</t>
-  </si>
-  <si>
-    <t>Romeral - Los Guaicos</t>
-  </si>
-  <si>
-    <t>Los Niches</t>
-  </si>
-  <si>
-    <t>Villa Prat - Sagrada Familia</t>
-  </si>
-  <si>
-    <t>Sol de Septiembre - Manuel Rodríguez</t>
-  </si>
-  <si>
-    <t>Feria - Mall - Terminal</t>
-  </si>
-  <si>
-    <t>Guaiquillo - Aguas Negras</t>
-  </si>
-  <si>
-    <t>Hospital - Alameda - Mataquito</t>
-  </si>
-  <si>
-    <t>Rauco - Comalle</t>
-  </si>
-  <si>
-    <t>Itahue Molina Estación</t>
-  </si>
-  <si>
-    <t>El Boldo</t>
-  </si>
-  <si>
-    <t>Bombero Garrido - Vaticano</t>
-  </si>
-  <si>
-    <t>La Montaña - Teno - Viluco</t>
-  </si>
-  <si>
-    <t>Santa Fe</t>
-  </si>
-  <si>
-    <t>Aguas Negras</t>
-  </si>
-  <si>
-    <t>Teno - Arboleda</t>
-  </si>
-  <si>
-    <t>Sarmiento - Rauquen</t>
-  </si>
-  <si>
-    <t>Molina Centro Porvenir</t>
-  </si>
-  <si>
-    <t>Bombero Garrido - Tutuquen</t>
-  </si>
-  <si>
-    <t>Santa Lucia - Santos Martínez</t>
-  </si>
-  <si>
-    <t>CURICÓ</t>
-  </si>
-  <si>
-    <t>Auditor : SAMUEL INOSTROZA NAVARRO</t>
-  </si>
-  <si>
-    <t>Linares: Obispo Camus - Yerbas Buenas</t>
-  </si>
-  <si>
-    <t>Auditor : CRISTIAN LIZAMA VERGARA</t>
-  </si>
-  <si>
-    <t>SAN FDO</t>
-  </si>
-  <si>
-    <t>ANGOSTURA -  18 DE SEPTIEMBRE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">APALTA - PANIAHUE </t>
-  </si>
-  <si>
-    <t>AUQUINCO - PUJILLAY</t>
-  </si>
-  <si>
-    <t>CALLEJONES - NANCAGUA</t>
-  </si>
-  <si>
-    <t>CHEPICA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHEPICA - LAS ALAMEDAS </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHEPICA - QUINAHUE </t>
-  </si>
-  <si>
-    <t>CHIMBARONGO  CENTRO</t>
-  </si>
-  <si>
-    <t>CHIMBARONGO CENTRO PTE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHIMBARONGO NORTE </t>
-  </si>
-  <si>
-    <t>CHIMBARONGO NORTE -CENTRO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHIMBARONGO SUR </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CODEGUA - PEOR ES NADA </t>
-  </si>
-  <si>
-    <t>CUNACO- CRUCE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL HHUIQUE - PERALILLO </t>
-  </si>
-  <si>
-    <t>LOLOL - LA LAJUELA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARCGIHUE </t>
-  </si>
-  <si>
-    <t>NANCAGUA -CENTRO</t>
-  </si>
-  <si>
-    <t>NANCAGUA - SAN GREGORIO</t>
-  </si>
-  <si>
-    <t>PAREDONES - LOLOL</t>
-  </si>
-  <si>
-    <t>PERALILLO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PICHILEMU -ALCONES </t>
-  </si>
-  <si>
-    <t>POICHILEMU - AV.CAHUIL</t>
-  </si>
-  <si>
-    <t>PICHILEMU - CENTRO</t>
-  </si>
-  <si>
-    <t>PICHILEMU - COSTANERA</t>
-  </si>
-  <si>
-    <t>PICHILEMU - INFIERNILLO</t>
-  </si>
-  <si>
-    <t>PICHILEMU - ORIENTE</t>
-  </si>
-  <si>
-    <t>PLACILLA</t>
-  </si>
-  <si>
-    <t>POBLACION - PERALILLO</t>
-  </si>
-  <si>
-    <t>PUENTE NEGRO - AGUA BUENA</t>
-  </si>
-  <si>
-    <t>PUMANQUE - NILAHUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROMA - MIRAFLORES -POLONIA </t>
-  </si>
-  <si>
-    <t>ROMERAL - SAN JUAN - TINGURIRICA</t>
-  </si>
-  <si>
-    <t>SAN FDO. - CENTINELA</t>
-  </si>
-  <si>
-    <t>SAN FDO. - CENTRO</t>
-  </si>
-  <si>
-    <t>SAN FDO. CENTRO 2</t>
-  </si>
-  <si>
-    <t>SAN FDO. CENTRO - PLAZA</t>
-  </si>
-  <si>
-    <t>SAN FDO. - MANSO DE VELASCO</t>
-  </si>
-  <si>
-    <t>SAN FDO, - GABRIELA MISTRAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAN FDO. - INDEPENDENCIA </t>
-  </si>
-  <si>
-    <t>SAN FDO. - NOR PONIENTE</t>
-  </si>
-  <si>
-    <t>SAN FDO. - ORIENTE</t>
-  </si>
-  <si>
-    <t>SAN FDO.  -SAN HERNAN</t>
-  </si>
-  <si>
-    <t>SAN FDO SUR</t>
-  </si>
-  <si>
-    <t>SAN  FDO. - SUR PONIENTE</t>
-  </si>
-  <si>
-    <t>SAN FDO. SUR PONIENTE 2</t>
-  </si>
-  <si>
-    <t>SAN FDO. TERMINAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STA CRUZ  - AV. ERRAZURIZ </t>
-  </si>
-  <si>
-    <t>STA CRUZ - BARREALES - PALMILLA</t>
-  </si>
-  <si>
-    <t>SATA .CRUZ ORIENTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STA CRUZ PONIENTE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">STA CRUZ SUR </t>
-  </si>
-  <si>
-    <t xml:space="preserve">STA CRUZ TERMINAL </t>
-  </si>
-  <si>
-    <t xml:space="preserve">VILLA ALEGRE - LA TUNA </t>
-  </si>
-  <si>
-    <t>CANT</t>
+    <t>Brilla el Sol, Daniel Rebolledo</t>
+  </si>
+  <si>
+    <t>activo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mayo </t>
+  </si>
+  <si>
+    <t>junio</t>
+  </si>
+  <si>
+    <t>julio</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -731,8 +747,15 @@
       <family val="2"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -751,6 +774,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -764,7 +793,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -781,6 +810,12 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -796,10 +831,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1636,16 +1667,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B1:D46"/>
+  <dimension ref="B1:E46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" customWidth="1"/>
     <col min="2" max="2" width="3.88671875" customWidth="1"/>
     <col min="3" max="3" width="33" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.88671875" style="1"/>
+    <col min="5" max="5" width="11.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1" s="2"/>
       <c r="C1" s="2" t="s">
         <v>52</v>
@@ -1654,10 +1686,10 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6"/>
       <c r="C3" s="6" t="s">
         <v>48</v>
@@ -1666,180 +1698,184 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="8">
+        <v>58</v>
+      </c>
+      <c r="E4" s="9">
+        <f>SUM(D4:D24)</f>
+        <v>1491</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="8">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" s="8">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" s="8">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D8" s="8">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B5">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B9">
         <v>2</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C9" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D9" s="8">
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" s="1">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="1">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="1">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B9">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="1">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>7</v>
       </c>
       <c r="C10" t="s">
         <v>59</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="8">
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>8</v>
       </c>
       <c r="C11" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="8">
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" s="8">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="8">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="8">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="8">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B16">
         <v>9</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C16" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D16" s="8">
         <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13">
-        <v>10</v>
-      </c>
-      <c r="C13" t="s">
-        <v>62</v>
-      </c>
-      <c r="D13" s="1">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14">
-        <v>11</v>
-      </c>
-      <c r="C14" t="s">
-        <v>63</v>
-      </c>
-      <c r="D14" s="1">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15">
-        <v>12</v>
-      </c>
-      <c r="C15" t="s">
-        <v>64</v>
-      </c>
-      <c r="D15" s="1">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16">
-        <v>13</v>
-      </c>
-      <c r="C16" t="s">
-        <v>65</v>
-      </c>
-      <c r="D16" s="1">
-        <v>60</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B17">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>66</v>
-      </c>
-      <c r="D17" s="1">
-        <v>60</v>
+        <v>62</v>
+      </c>
+      <c r="D17" s="8">
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B18">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
-      </c>
-      <c r="D18" s="1">
-        <v>58</v>
+        <v>57</v>
+      </c>
+      <c r="D18" s="8">
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B19">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
-      </c>
-      <c r="D19" s="1">
         <v>58</v>
+      </c>
+      <c r="D19" s="8">
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.3">
@@ -1849,7 +1885,7 @@
       <c r="C20" t="s">
         <v>69</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="8">
         <v>80</v>
       </c>
     </row>
@@ -1860,293 +1896,298 @@
       <c r="C21" t="s">
         <v>70</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="8">
         <v>80</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B22">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C22" t="s">
-        <v>71</v>
-      </c>
-      <c r="D22" s="1">
-        <v>180</v>
+        <v>78</v>
+      </c>
+      <c r="D22" s="8">
+        <v>90</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B23">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>72</v>
-      </c>
-      <c r="D23" s="1">
-        <v>180</v>
+        <v>5</v>
+      </c>
+      <c r="D23" s="8">
+        <v>90</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B24">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C24" t="s">
-        <v>73</v>
-      </c>
-      <c r="D24" s="1">
-        <v>175</v>
+        <v>75</v>
+      </c>
+      <c r="D24" s="8">
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B25">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>74</v>
-      </c>
-      <c r="D25" s="1">
-        <v>175</v>
+        <v>76</v>
+      </c>
+      <c r="D25" s="8">
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B26">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>75</v>
-      </c>
-      <c r="D26" s="1">
+        <v>30</v>
+      </c>
+      <c r="D26" s="8">
         <v>95</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B27">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="1">
+        <v>77</v>
+      </c>
+      <c r="D27" s="8">
         <v>95</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B28">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C28" t="s">
-        <v>30</v>
-      </c>
-      <c r="D28" s="1">
-        <v>95</v>
+        <v>79</v>
+      </c>
+      <c r="D28" s="8">
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B29">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D29" s="1">
-        <v>95</v>
+        <v>80</v>
+      </c>
+      <c r="D29" s="8">
+        <v>145</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B30">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="C30" t="s">
-        <v>78</v>
-      </c>
-      <c r="D30" s="1">
-        <v>90</v>
+        <v>87</v>
+      </c>
+      <c r="D30" s="8">
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B31">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C31" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="1">
-        <v>90</v>
+        <v>88</v>
+      </c>
+      <c r="D31" s="8">
+        <v>145</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B32">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32" t="s">
-        <v>79</v>
-      </c>
-      <c r="D32" s="1">
-        <v>145</v>
+        <v>81</v>
+      </c>
+      <c r="D32" s="8">
+        <v>160</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B33">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>80</v>
-      </c>
-      <c r="D33" s="1">
-        <v>145</v>
+        <v>82</v>
+      </c>
+      <c r="D33" s="8">
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B34">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C34" t="s">
-        <v>81</v>
-      </c>
-      <c r="D34" s="1">
+        <v>93</v>
+      </c>
+      <c r="D34" s="8">
         <v>160</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B35">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C35" t="s">
-        <v>82</v>
-      </c>
-      <c r="D35" s="1">
-        <v>160</v>
+        <v>85</v>
+      </c>
+      <c r="D35" s="8">
+        <v>170</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B36">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C36" t="s">
-        <v>83</v>
-      </c>
-      <c r="D36" s="1">
-        <v>275</v>
+        <v>86</v>
+      </c>
+      <c r="D36" s="8">
+        <v>170</v>
       </c>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B37">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="C37" t="s">
-        <v>84</v>
-      </c>
-      <c r="D37" s="1">
-        <v>275</v>
+        <v>73</v>
+      </c>
+      <c r="D37" s="8">
+        <v>175</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B38">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="C38" t="s">
-        <v>85</v>
-      </c>
-      <c r="D38" s="1">
-        <v>170</v>
+        <v>74</v>
+      </c>
+      <c r="D38" s="8">
+        <v>175</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B39">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="C39" t="s">
-        <v>86</v>
-      </c>
-      <c r="D39" s="1">
-        <v>170</v>
+        <v>71</v>
+      </c>
+      <c r="D39" s="8">
+        <v>180</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B40">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="C40" t="s">
-        <v>87</v>
-      </c>
-      <c r="D40" s="1">
-        <v>145</v>
+        <v>72</v>
+      </c>
+      <c r="D40" s="8">
+        <v>180</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B41">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>88</v>
-      </c>
-      <c r="D41" s="1">
-        <v>145</v>
+        <v>89</v>
+      </c>
+      <c r="D41" s="8">
+        <v>220</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B42">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
-        <v>89</v>
-      </c>
-      <c r="D42" s="1">
+        <v>90</v>
+      </c>
+      <c r="D42" s="8">
         <v>220</v>
       </c>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B43">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C43" t="s">
-        <v>90</v>
-      </c>
-      <c r="D43" s="1">
-        <v>220</v>
+        <v>91</v>
+      </c>
+      <c r="D43" s="8">
+        <v>260</v>
       </c>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B44">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C44" t="s">
-        <v>91</v>
-      </c>
-      <c r="D44" s="1">
+        <v>92</v>
+      </c>
+      <c r="D44" s="8">
         <v>260</v>
       </c>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B45">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="C45" t="s">
-        <v>92</v>
-      </c>
-      <c r="D45" s="1">
-        <v>260</v>
+        <v>83</v>
+      </c>
+      <c r="D45" s="8">
+        <v>275</v>
       </c>
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B46">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="C46" t="s">
-        <v>93</v>
-      </c>
-      <c r="D46" s="1">
-        <v>160</v>
+        <v>84</v>
+      </c>
+      <c r="D46" s="8">
+        <v>275</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B3:D46" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:D46">
+      <sortCondition ref="D3:D46"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B1:D42"/>
+  <dimension ref="B1:E46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" customWidth="1"/>
@@ -2155,7 +2196,7 @@
     <col min="4" max="4" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1" s="2"/>
       <c r="C1" s="2" t="s">
         <v>94</v>
@@ -2164,10 +2205,10 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6"/>
       <c r="C3" s="6" t="s">
         <v>48</v>
@@ -2175,8 +2216,11 @@
       <c r="D3" s="7" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E3" s="4" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>1</v>
       </c>
@@ -2187,7 +2231,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>2</v>
       </c>
@@ -2198,7 +2242,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>3</v>
       </c>
@@ -2208,8 +2252,11 @@
       <c r="D6" s="1">
         <v>62</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>4</v>
       </c>
@@ -2219,8 +2266,11 @@
       <c r="D7" s="1">
         <v>62</v>
       </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>5</v>
       </c>
@@ -2231,7 +2281,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>6</v>
       </c>
@@ -2242,7 +2292,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>7</v>
       </c>
@@ -2252,8 +2302,11 @@
       <c r="D10" s="1">
         <v>118</v>
       </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>8</v>
       </c>
@@ -2263,8 +2316,11 @@
       <c r="D11" s="1">
         <v>118</v>
       </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>9</v>
       </c>
@@ -2274,8 +2330,11 @@
       <c r="D12" s="1">
         <v>75</v>
       </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>10</v>
       </c>
@@ -2285,8 +2344,11 @@
       <c r="D13" s="1">
         <v>75</v>
       </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14">
         <v>11</v>
       </c>
@@ -2297,7 +2359,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15">
         <v>12</v>
       </c>
@@ -2308,7 +2370,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16">
         <v>13</v>
       </c>
@@ -2318,8 +2380,11 @@
       <c r="D16" s="1">
         <v>60</v>
       </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17">
         <v>14</v>
       </c>
@@ -2329,8 +2394,11 @@
       <c r="D17" s="1">
         <v>60</v>
       </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18">
         <v>15</v>
       </c>
@@ -2341,7 +2409,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19">
         <v>16</v>
       </c>
@@ -2352,29 +2420,35 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>17</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="11" t="s">
         <v>110</v>
       </c>
       <c r="D20" s="1">
         <v>86</v>
       </c>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>18</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="11" t="s">
         <v>111</v>
       </c>
       <c r="D21" s="1">
         <v>86</v>
       </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>19</v>
       </c>
@@ -2385,7 +2459,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>20</v>
       </c>
@@ -2396,7 +2470,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24">
         <v>21</v>
       </c>
@@ -2407,7 +2481,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25">
         <v>22</v>
       </c>
@@ -2418,192 +2492,212 @@
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26">
         <v>23</v>
       </c>
       <c r="C26" t="s">
-        <v>116</v>
+        <v>218</v>
       </c>
       <c r="D26" s="1">
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27">
         <v>24</v>
       </c>
       <c r="C27" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D27" s="1">
         <v>55</v>
       </c>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28">
         <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D28" s="1">
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29">
         <v>26</v>
       </c>
       <c r="C29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D29" s="1">
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30">
         <v>27</v>
       </c>
       <c r="C30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D30" s="1">
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31">
         <v>28</v>
       </c>
       <c r="C31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D31" s="1">
         <v>200</v>
       </c>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32">
         <v>29</v>
       </c>
       <c r="C32" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D32" s="1">
         <v>200</v>
       </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33">
         <v>30</v>
       </c>
       <c r="C33" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D33" s="1">
         <v>165</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34">
         <v>31</v>
       </c>
       <c r="C34" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D34" s="1">
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35">
         <v>32</v>
       </c>
       <c r="C35" t="s">
-        <v>124</v>
+        <v>219</v>
       </c>
       <c r="D35" s="1">
         <v>160</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36">
         <v>33</v>
       </c>
       <c r="C36" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D36" s="1">
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B37">
         <v>34</v>
       </c>
       <c r="C37" t="s">
-        <v>126</v>
+        <v>220</v>
       </c>
       <c r="D37" s="1">
         <v>130</v>
       </c>
     </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B38">
         <v>35</v>
       </c>
       <c r="C38" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D38" s="1">
         <v>220</v>
       </c>
     </row>
-    <row r="39" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B39">
         <v>36</v>
       </c>
       <c r="C39" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D39" s="1">
         <v>220</v>
       </c>
     </row>
-    <row r="40" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B40">
         <v>37</v>
       </c>
       <c r="C40" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D40" s="1">
         <v>160</v>
       </c>
     </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B41">
         <v>38</v>
       </c>
       <c r="C41" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D41" s="1">
         <v>160</v>
       </c>
     </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B42">
         <v>39</v>
       </c>
       <c r="C42" t="s">
-        <v>131</v>
+        <v>221</v>
       </c>
       <c r="D42" s="1">
         <v>150</v>
       </c>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B43">
+        <v>40</v>
+      </c>
+      <c r="C43" t="s">
+        <v>222</v>
+      </c>
+      <c r="D43" s="1">
+        <v>80</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E46" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2613,7 +2707,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B1:D34"/>
+  <dimension ref="B1:H35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" customWidth="1"/>
@@ -2622,21 +2716,21 @@
     <col min="4" max="4" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1" s="2"/>
       <c r="C1" s="4" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="2" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2" spans="2:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>48</v>
@@ -2644,352 +2738,551 @@
       <c r="D3" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="F3" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D4" s="1">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D5" s="1">
         <v>286</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D6" s="1">
+        <v>284</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="1">
+        <v>272</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B8">
         <v>3</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C8" t="s">
+        <v>130</v>
+      </c>
+      <c r="D8" s="1">
+        <v>249</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
         <v>134</v>
       </c>
-      <c r="D6" s="1">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>135</v>
-      </c>
-      <c r="D7" s="1">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>136</v>
-      </c>
-      <c r="D8" s="1">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B9">
+      <c r="D9" s="1">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B10">
         <v>6</v>
       </c>
-      <c r="C9" t="s">
-        <v>137</v>
-      </c>
-      <c r="D9" s="1">
+      <c r="C10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D10" s="1">
         <v>173</v>
       </c>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B10">
-        <v>7</v>
-      </c>
-      <c r="C10" t="s">
-        <v>138</v>
-      </c>
-      <c r="D10" s="1">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="F10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D11" s="1">
+        <v>149</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D12" s="1">
+        <v>148</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>14</v>
+      </c>
+      <c r="C13" t="s">
+        <v>140</v>
+      </c>
+      <c r="D13" s="1">
+        <v>142</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>146</v>
+      </c>
+      <c r="D14" s="1">
+        <v>142</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>13</v>
+      </c>
+      <c r="C15" t="s">
         <v>139</v>
       </c>
-      <c r="D11" s="1">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12">
-        <v>9</v>
-      </c>
-      <c r="C12" t="s">
-        <v>140</v>
-      </c>
-      <c r="D12" s="1">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13">
-        <v>10</v>
-      </c>
-      <c r="C13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D13" s="1">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14">
-        <v>11</v>
-      </c>
-      <c r="C14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D14" s="1">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15">
-        <v>12</v>
-      </c>
-      <c r="C15" t="s">
-        <v>142</v>
-      </c>
       <c r="D15" s="1">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="D16" s="1">
         <v>111</v>
       </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B17">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C17" t="s">
+        <v>137</v>
+      </c>
+      <c r="D17" s="1">
+        <v>108</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B18">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>138</v>
+      </c>
+      <c r="D18" s="1">
+        <v>108</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B19">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
+        <v>147</v>
+      </c>
+      <c r="D19" s="1">
+        <v>102</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B20">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
+        <v>136</v>
+      </c>
+      <c r="D20" s="1">
+        <v>98</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <v>16</v>
+      </c>
+      <c r="C21" t="s">
+        <v>142</v>
+      </c>
+      <c r="D21" s="1">
+        <v>98</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B22">
+        <v>30</v>
+      </c>
+      <c r="C22" t="s">
+        <v>156</v>
+      </c>
+      <c r="D22" s="1">
+        <v>98</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <v>27</v>
+      </c>
+      <c r="C23" t="s">
+        <v>153</v>
+      </c>
+      <c r="D23" s="1">
+        <v>94</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B24">
+        <v>23</v>
+      </c>
+      <c r="C24" t="s">
+        <v>149</v>
+      </c>
+      <c r="D24" s="1">
+        <v>78</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B25">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>154</v>
+      </c>
+      <c r="D25" s="1">
+        <v>78</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B26">
+        <v>25</v>
+      </c>
+      <c r="C26" t="s">
+        <v>151</v>
+      </c>
+      <c r="D26" s="1">
+        <v>69</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B27">
+        <v>31</v>
+      </c>
+      <c r="C27" t="s">
+        <v>157</v>
+      </c>
+      <c r="D27" s="1">
+        <v>69</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B28">
+        <v>19</v>
+      </c>
+      <c r="C28" t="s">
+        <v>145</v>
+      </c>
+      <c r="D28" s="1">
+        <v>68</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B29">
+        <v>18</v>
+      </c>
+      <c r="C29" t="s">
         <v>144</v>
       </c>
-      <c r="D17" s="1">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18">
-        <v>15</v>
-      </c>
-      <c r="C18" t="s">
-        <v>145</v>
-      </c>
-      <c r="D18" s="1">
+      <c r="D29" s="1">
+        <v>63</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B30">
+        <v>22</v>
+      </c>
+      <c r="C30" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19">
-        <v>16</v>
-      </c>
-      <c r="C19" t="s">
-        <v>146</v>
-      </c>
-      <c r="D19" s="1">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20">
+      <c r="D30" s="1">
+        <v>59</v>
+      </c>
+      <c r="F30">
+        <v>1</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B31">
+        <v>26</v>
+      </c>
+      <c r="C31" t="s">
+        <v>152</v>
+      </c>
+      <c r="D31" s="1">
+        <v>59</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31">
+        <v>1</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B32">
+        <v>8</v>
+      </c>
+      <c r="C32" t="s">
+        <v>135</v>
+      </c>
+      <c r="D32" s="1">
+        <v>47</v>
+      </c>
+      <c r="G32">
+        <v>1</v>
+      </c>
+      <c r="H32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B33">
+        <v>11</v>
+      </c>
+      <c r="C33" t="s">
+        <v>66</v>
+      </c>
+      <c r="D33" s="1">
+        <v>47</v>
+      </c>
+      <c r="F33">
+        <v>1</v>
+      </c>
+      <c r="G33">
+        <v>1</v>
+      </c>
+      <c r="H33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B34">
         <v>17</v>
       </c>
-      <c r="C20" t="s">
-        <v>147</v>
-      </c>
-      <c r="D20" s="1">
+      <c r="C34" t="s">
+        <v>143</v>
+      </c>
+      <c r="D34" s="1">
         <v>47</v>
       </c>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B21">
-        <v>18</v>
-      </c>
-      <c r="C21" t="s">
-        <v>148</v>
-      </c>
-      <c r="D21" s="1">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B22">
-        <v>19</v>
-      </c>
-      <c r="C22" t="s">
-        <v>149</v>
-      </c>
-      <c r="D22" s="1">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B23">
-        <v>20</v>
-      </c>
-      <c r="C23" t="s">
-        <v>150</v>
-      </c>
-      <c r="D23" s="1">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B24">
-        <v>21</v>
-      </c>
-      <c r="C24" t="s">
-        <v>151</v>
-      </c>
-      <c r="D24" s="1">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B25">
+      <c r="G34">
+        <v>1</v>
+      </c>
+      <c r="H34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G35">
+        <f xml:space="preserve"> SUM(G4:G34)</f>
         <v>22</v>
       </c>
-      <c r="C25" t="s">
-        <v>152</v>
-      </c>
-      <c r="D25" s="1">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B26">
-        <v>23</v>
-      </c>
-      <c r="C26" t="s">
-        <v>153</v>
-      </c>
-      <c r="D26" s="1">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B27">
-        <v>24</v>
-      </c>
-      <c r="C27" t="s">
-        <v>154</v>
-      </c>
-      <c r="D27" s="1">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B28">
-        <v>25</v>
-      </c>
-      <c r="C28" t="s">
-        <v>155</v>
-      </c>
-      <c r="D28" s="1">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B29">
-        <v>26</v>
-      </c>
-      <c r="C29" t="s">
-        <v>156</v>
-      </c>
-      <c r="D29" s="1">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B30">
-        <v>27</v>
-      </c>
-      <c r="C30" t="s">
-        <v>157</v>
-      </c>
-      <c r="D30" s="1">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B31">
-        <v>28</v>
-      </c>
-      <c r="C31" t="s">
-        <v>158</v>
-      </c>
-      <c r="D31" s="1">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B32">
-        <v>29</v>
-      </c>
-      <c r="C32" t="s">
-        <v>159</v>
-      </c>
-      <c r="D32" s="1">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B33">
-        <v>30</v>
-      </c>
-      <c r="C33" t="s">
-        <v>160</v>
-      </c>
-      <c r="D33" s="1">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B34">
-        <v>31</v>
-      </c>
-      <c r="C34" t="s">
-        <v>161</v>
-      </c>
-      <c r="D34" s="1">
-        <v>69</v>
+      <c r="H35">
+        <f>SUM(H4:H34)</f>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B3:D34" xr:uid="{00000000-0009-0000-0000-000003000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:D34">
-      <sortCondition ref="B3:B34"/>
+  <autoFilter ref="B3:G34" xr:uid="{00000000-0001-0000-0300-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:G34">
+      <sortCondition descending="1" ref="D3:D34"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3011,10 +3304,10 @@
     <row r="1" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B1" s="2"/>
       <c r="C1" s="4" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.3">
@@ -3024,7 +3317,7 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>48</v>
@@ -3038,7 +3331,7 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D4">
         <v>51</v>
@@ -3049,7 +3342,7 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D5">
         <v>112</v>
@@ -3060,7 +3353,7 @@
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D6">
         <v>137</v>
@@ -3071,7 +3364,7 @@
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D7">
         <v>82</v>
@@ -3082,7 +3375,7 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D8">
         <v>118</v>
@@ -3093,7 +3386,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D9">
         <v>129</v>
@@ -3104,7 +3397,7 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D10">
         <v>121</v>
@@ -3115,7 +3408,7 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D11">
         <v>65</v>
@@ -3126,7 +3419,7 @@
         <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D12">
         <v>65</v>
@@ -3137,7 +3430,7 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D13">
         <v>61</v>
@@ -3148,7 +3441,7 @@
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D14">
         <v>61</v>
@@ -3159,7 +3452,7 @@
         <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D15">
         <v>68</v>
@@ -3170,7 +3463,7 @@
         <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D16">
         <v>108</v>
@@ -3181,7 +3474,7 @@
         <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D17">
         <v>125</v>
@@ -3192,7 +3485,7 @@
         <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D18">
         <v>178</v>
@@ -3203,7 +3496,7 @@
         <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D19">
         <v>188</v>
@@ -3214,7 +3507,7 @@
         <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D20">
         <v>190</v>
@@ -3225,7 +3518,7 @@
         <v>18</v>
       </c>
       <c r="C21" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D21">
         <v>75</v>
@@ -3236,7 +3529,7 @@
         <v>19</v>
       </c>
       <c r="C22" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D22">
         <v>75</v>
@@ -3247,7 +3540,7 @@
         <v>20</v>
       </c>
       <c r="C23" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D23">
         <v>244</v>
@@ -3258,7 +3551,7 @@
         <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D24">
         <v>150</v>
@@ -3269,7 +3562,7 @@
         <v>22</v>
       </c>
       <c r="C25" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D25">
         <v>280</v>
@@ -3280,7 +3573,7 @@
         <v>23</v>
       </c>
       <c r="C26" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D26">
         <v>295</v>
@@ -3291,7 +3584,7 @@
         <v>24</v>
       </c>
       <c r="C27" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D27">
         <v>282</v>
@@ -3302,7 +3595,7 @@
         <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D28">
         <v>292</v>
@@ -3313,7 +3606,7 @@
         <v>26</v>
       </c>
       <c r="C29" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D29">
         <v>305</v>
@@ -3324,7 +3617,7 @@
         <v>27</v>
       </c>
       <c r="C30" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D30">
         <v>286</v>
@@ -3335,7 +3628,7 @@
         <v>28</v>
       </c>
       <c r="C31" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D31">
         <v>67</v>
@@ -3346,7 +3639,7 @@
         <v>29</v>
       </c>
       <c r="C32" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="D32">
         <v>178</v>
@@ -3357,7 +3650,7 @@
         <v>30</v>
       </c>
       <c r="C33" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D33">
         <v>72</v>
@@ -3368,7 +3661,7 @@
         <v>31</v>
       </c>
       <c r="C34" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D34">
         <v>238</v>
@@ -3379,7 +3672,7 @@
         <v>32</v>
       </c>
       <c r="C35" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D35">
         <v>54</v>
@@ -3390,7 +3683,7 @@
         <v>33</v>
       </c>
       <c r="C36" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D36">
         <v>92</v>
@@ -3401,7 +3694,7 @@
         <v>34</v>
       </c>
       <c r="C37" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D37">
         <v>35</v>
@@ -3412,7 +3705,7 @@
         <v>35</v>
       </c>
       <c r="C38" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D38">
         <v>25</v>
@@ -3423,7 +3716,7 @@
         <v>36</v>
       </c>
       <c r="C39" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D39">
         <v>25</v>
@@ -3434,7 +3727,7 @@
         <v>37</v>
       </c>
       <c r="C40" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D40">
         <v>31</v>
@@ -3445,7 +3738,7 @@
         <v>38</v>
       </c>
       <c r="C41" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D41">
         <v>25</v>
@@ -3456,7 +3749,7 @@
         <v>39</v>
       </c>
       <c r="C42" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D42">
         <v>32</v>
@@ -3467,7 +3760,7 @@
         <v>40</v>
       </c>
       <c r="C43" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D43">
         <v>33</v>
@@ -3478,7 +3771,7 @@
         <v>41</v>
       </c>
       <c r="C44" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D44">
         <v>33</v>
@@ -3489,7 +3782,7 @@
         <v>42</v>
       </c>
       <c r="C45" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="D45">
         <v>34</v>
@@ -3500,7 +3793,7 @@
         <v>43</v>
       </c>
       <c r="C46" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D46">
         <v>33</v>
@@ -3515,7 +3808,7 @@
         <v>44</v>
       </c>
       <c r="C47" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D47">
         <v>35</v>
@@ -3526,7 +3819,7 @@
         <v>45</v>
       </c>
       <c r="C48" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="D48">
         <v>35</v>
@@ -3541,7 +3834,7 @@
         <v>46</v>
       </c>
       <c r="C49" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D49">
         <v>35</v>
@@ -3552,7 +3845,7 @@
         <v>47</v>
       </c>
       <c r="C50" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="D50">
         <v>25</v>
@@ -3563,7 +3856,7 @@
         <v>48</v>
       </c>
       <c r="C51" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D51">
         <v>104</v>
@@ -3574,7 +3867,7 @@
         <v>49</v>
       </c>
       <c r="C52" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="D52">
         <v>158</v>
@@ -3585,7 +3878,7 @@
         <v>50</v>
       </c>
       <c r="C53" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D53">
         <v>110</v>
@@ -3596,7 +3889,7 @@
         <v>51</v>
       </c>
       <c r="C54" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D54">
         <v>104</v>
@@ -3607,7 +3900,7 @@
         <v>52</v>
       </c>
       <c r="C55" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D55">
         <v>115</v>
@@ -3618,7 +3911,7 @@
         <v>53</v>
       </c>
       <c r="C56" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D56">
         <v>62</v>
@@ -3629,7 +3922,7 @@
         <v>54</v>
       </c>
       <c r="C57" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D57">
         <v>62</v>

</xml_diff>